<commit_message>
Add SOH report for 2026-10-02
</commit_message>
<xml_diff>
--- a/reports/SOH_01_10_2026.xlsx
+++ b/reports/SOH_01_10_2026.xlsx
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>21000</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>21000</v>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>25000</v>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>48000</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>10500</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -1931,24 +1931,24 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>6972731711385</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AWB12-012</t>
+          <t>AWB18-018</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Pull Up Pants 12 Medium (2 Pcs)</t>
+          <t>AIWIBI Baby Pull Up Night Pants 18 XXXL (2Pcs)</t>
         </is>
       </c>
       <c r="D54" s="2" t="n">
-        <v>1302</v>
+        <v>85</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>3700</v>
+        <v>5000</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -1959,24 +1959,24 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>6972731711477</t>
+          <t>6972731711385</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AWB12-02</t>
+          <t>AWB01-014</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Pull Up Pants 12 Medium (5* 48 Pcs)</t>
+          <t>AIWIBI Baby Pull Up Pants  Extra Large (2pcs)</t>
         </is>
       </c>
       <c r="D55" s="2" t="n">
-        <v>604</v>
+        <v>974</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>51000</v>
+        <v>4100</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -1992,19 +1992,19 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AWB01-014</t>
+          <t>AWB12-012</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Pull Up Pants  Extra Large (2pcs)</t>
+          <t>AIWIBI Baby Pull Up Pants 12 Medium (2 Pcs)</t>
         </is>
       </c>
       <c r="D56" s="2" t="n">
-        <v>974</v>
+        <v>1302</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>4100</v>
+        <v>3700</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2015,21 +2015,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>6972731711484</t>
+          <t>6972731711477</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AWB12-01</t>
+          <t>AWB12-02</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Pull Up Pants 12 Small (5* 52 Pcs)</t>
+          <t>AIWIBI Baby Pull Up Pants 12 Medium (5* 48 Pcs)</t>
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>2</v>
+        <v>604</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2043,24 +2043,24 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6972731711484</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>AWB18-018</t>
+          <t>AWB12-01</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Pull Up Night Pants 18 XXXL (2Pcs)</t>
+          <t>AIWIBI Baby Pull Up Pants 12 Small (5* 52 Pcs)</t>
         </is>
       </c>
       <c r="D58" s="2" t="n">
-        <v>85</v>
+        <v>2</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>5000</v>
+        <v>51000</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>26500</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>4000</v>
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E107" s="3" t="n">
         <v>1</v>
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>5010</v>
+        <v>4986</v>
       </c>
       <c r="E126" s="3" t="n">
         <v>2500</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>681</v>
+        <v>657</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E155" s="3" t="n">
         <v>1</v>
@@ -4797,7 +4797,7 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="E156" s="3" t="n">
         <v>26000</v>
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="E159" s="3" t="n">
         <v>1</v>
@@ -5125,7 +5125,7 @@
         </is>
       </c>
       <c r="D168" s="2" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E168" s="3" t="n">
         <v>1</v>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>840</v>
+        <v>825</v>
       </c>
       <c r="E174" s="3" t="n">
         <v>13500</v>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E177" s="3" t="n">
         <v>1</v>
@@ -6373,7 +6373,7 @@
         </is>
       </c>
       <c r="D214" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E214" s="3" t="n">
         <v>0</v>
@@ -7581,7 +7581,7 @@
         </is>
       </c>
       <c r="D259" s="2" t="n">
-        <v>696</v>
+        <v>684</v>
       </c>
       <c r="E259" s="3" t="n">
         <v>6350</v>
@@ -8085,7 +8085,7 @@
         </is>
       </c>
       <c r="D277" s="2" t="n">
-        <v>1483</v>
+        <v>1471</v>
       </c>
       <c r="E277" s="3" t="n">
         <v>3708</v>
@@ -12986,7 +12986,7 @@
         </is>
       </c>
       <c r="D452" s="2" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E452" s="3" t="n">
         <v>6183</v>
@@ -13742,7 +13742,7 @@
         </is>
       </c>
       <c r="D479" s="2" t="n">
-        <v>1821</v>
+        <v>1797</v>
       </c>
       <c r="E479" s="3" t="n">
         <v>15262</v>
@@ -14148,24 +14148,24 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>9333527429780</t>
+          <t>9333527392299</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>AG2084</t>
+          <t>KC0341</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>COOLING EYE MASK 20 X 9CM</t>
+          <t>COOKIE BAKING TRAY LGE 43x29cm</t>
         </is>
       </c>
       <c r="D494" s="2" t="n">
-        <v>157</v>
+        <v>7</v>
       </c>
       <c r="E494" s="3" t="n">
-        <v>17322</v>
+        <v>12979</v>
       </c>
       <c r="F494" t="inlineStr">
         <is>
@@ -14176,24 +14176,24 @@
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>9333527392299</t>
+          <t>9333527429780</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>KC0341</t>
+          <t>AG2084</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>COOKIE BAKING TRAY LGE 43x29cm</t>
+          <t>COOLING EYE MASK 20 X 9CM</t>
         </is>
       </c>
       <c r="D495" s="2" t="n">
-        <v>7</v>
+        <v>157</v>
       </c>
       <c r="E495" s="3" t="n">
-        <v>12979</v>
+        <v>17322</v>
       </c>
       <c r="F495" t="inlineStr">
         <is>
@@ -14498,7 +14498,7 @@
         </is>
       </c>
       <c r="D506" s="2" t="n">
-        <v>1317</v>
+        <v>1305</v>
       </c>
       <c r="E506" s="3" t="n">
         <v>8446</v>
@@ -15114,7 +15114,7 @@
         </is>
       </c>
       <c r="D528" s="2" t="n">
-        <v>475</v>
+        <v>469</v>
       </c>
       <c r="E528" s="3" t="n">
         <v>22302</v>
@@ -15170,7 +15170,7 @@
         </is>
       </c>
       <c r="D530" s="2" t="n">
-        <v>412</v>
+        <v>400</v>
       </c>
       <c r="E530" s="3" t="n">
         <v>12816</v>
@@ -17551,7 +17551,7 @@
         </is>
       </c>
       <c r="D615" s="2" t="n">
-        <v>4475</v>
+        <v>4439</v>
       </c>
       <c r="E615" s="3" t="n">
         <v>10251</v>
@@ -18545,24 +18545,24 @@
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
-          <t>9333527043160</t>
+          <t>9333527037961</t>
         </is>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>OX0156</t>
+          <t>BC0079</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
         <is>
-          <t>FROG WINDOW THERMOMETER</t>
+          <t>FREEZER BAG 100PK ON ROLL 20X3</t>
         </is>
       </c>
       <c r="D651" s="2" t="n">
-        <v>0</v>
+        <v>898</v>
       </c>
       <c r="E651" s="3" t="n">
-        <v>15693</v>
+        <v>6417</v>
       </c>
       <c r="F651" t="inlineStr">
         <is>
@@ -18573,24 +18573,24 @@
     <row r="652">
       <c r="A652" t="inlineStr">
         <is>
-          <t>9333527731814</t>
+          <t>9333527469465</t>
         </is>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>TN2183</t>
+          <t>BC0476</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>FROG/SPIDER SQUEEZE BALL 2ASST</t>
+          <t>FREEZER BAGS 30PK</t>
         </is>
       </c>
       <c r="D652" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E652" s="3" t="n">
-        <v>12665</v>
+        <v>9808</v>
       </c>
       <c r="F652" t="inlineStr">
         <is>
@@ -18601,24 +18601,24 @@
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>9333527469465</t>
+          <t>9333527477019</t>
         </is>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>BC0476</t>
+          <t>BC0480</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>FREEZER BAGS 30PK</t>
+          <t>FREEZER DOUBLE ZIP BAGS 24PK</t>
         </is>
       </c>
       <c r="D653" s="2" t="n">
-        <v>0</v>
+        <v>1213</v>
       </c>
       <c r="E653" s="3" t="n">
-        <v>9808</v>
+        <v>11078</v>
       </c>
       <c r="F653" t="inlineStr">
         <is>
@@ -18629,24 +18629,24 @@
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>9333527477019</t>
+          <t>9333527043160</t>
         </is>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>BC0480</t>
+          <t>OX0156</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>FREEZER DOUBLE ZIP BAGS 24PK</t>
+          <t>FROG WINDOW THERMOMETER</t>
         </is>
       </c>
       <c r="D654" s="2" t="n">
-        <v>1213</v>
+        <v>0</v>
       </c>
       <c r="E654" s="3" t="n">
-        <v>11078</v>
+        <v>15693</v>
       </c>
       <c r="F654" t="inlineStr">
         <is>
@@ -18657,24 +18657,24 @@
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
-          <t>9333527037961</t>
+          <t>9333527731814</t>
         </is>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>BC0079</t>
+          <t>TN2183</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>FREEZER BAG 100PK ON ROLL 20X3</t>
+          <t>FROG/SPIDER SQUEEZE BALL 2ASST</t>
         </is>
       </c>
       <c r="D655" s="2" t="n">
-        <v>898</v>
+        <v>0</v>
       </c>
       <c r="E655" s="3" t="n">
-        <v>6417</v>
+        <v>12665</v>
       </c>
       <c r="F655" t="inlineStr">
         <is>
@@ -19329,24 +19329,24 @@
     <row r="679">
       <c r="A679" t="inlineStr">
         <is>
-          <t>8409730015070</t>
+          <t>8409730014646</t>
         </is>
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>SC0010</t>
+          <t>SC0003</t>
         </is>
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>GIFT BAG HOLOGRAPH 33X42CM XLG</t>
+          <t>GIFT BAG HOLOGRAPH 11X14CM SM</t>
         </is>
       </c>
       <c r="D679" s="2" t="n">
-        <v>158</v>
+        <v>354</v>
       </c>
       <c r="E679" s="3" t="n">
-        <v>6039</v>
+        <v>2338</v>
       </c>
       <c r="F679" t="inlineStr">
         <is>
@@ -19357,24 +19357,24 @@
     <row r="680">
       <c r="A680" t="inlineStr">
         <is>
-          <t>8409730014400</t>
+          <t>8409730014578</t>
         </is>
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>SC0001</t>
+          <t>SC0002</t>
         </is>
       </c>
       <c r="C680" t="inlineStr">
         <is>
-          <t>GIFT BAG HOLOGRAPH 26X32CM LG</t>
+          <t>GIFT BAG HOLOGRAPH 18X23CM MED1920</t>
         </is>
       </c>
       <c r="D680" s="2" t="n">
-        <v>597</v>
+        <v>324</v>
       </c>
       <c r="E680" s="3" t="n">
-        <v>2870</v>
+        <v>1920</v>
       </c>
       <c r="F680" t="inlineStr">
         <is>
@@ -19385,24 +19385,24 @@
     <row r="681">
       <c r="A681" t="inlineStr">
         <is>
-          <t>4894158140598</t>
+          <t>8409730014400</t>
         </is>
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>XM5589</t>
+          <t>SC0001</t>
         </is>
       </c>
       <c r="C681" t="inlineStr">
         <is>
-          <t>GIFT BAG NON-WOVEN PRINTED Asst</t>
+          <t>GIFT BAG HOLOGRAPH 26X32CM LG</t>
         </is>
       </c>
       <c r="D681" s="2" t="n">
-        <v>9</v>
+        <v>597</v>
       </c>
       <c r="E681" s="3" t="n">
-        <v>8656</v>
+        <v>2870</v>
       </c>
       <c r="F681" t="inlineStr">
         <is>
@@ -19413,24 +19413,24 @@
     <row r="682">
       <c r="A682" t="inlineStr">
         <is>
-          <t>8409730014646</t>
+          <t>8409730015070</t>
         </is>
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>SC0003</t>
+          <t>SC0010</t>
         </is>
       </c>
       <c r="C682" t="inlineStr">
         <is>
-          <t>GIFT BAG HOLOGRAPH 11X14CM SM</t>
+          <t>GIFT BAG HOLOGRAPH 33X42CM XLG</t>
         </is>
       </c>
       <c r="D682" s="2" t="n">
-        <v>354</v>
+        <v>158</v>
       </c>
       <c r="E682" s="3" t="n">
-        <v>2338</v>
+        <v>6039</v>
       </c>
       <c r="F682" t="inlineStr">
         <is>
@@ -19441,24 +19441,24 @@
     <row r="683">
       <c r="A683" t="inlineStr">
         <is>
-          <t>8409730014578</t>
+          <t>4894158140598</t>
         </is>
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>SC0002</t>
+          <t>XM5589</t>
         </is>
       </c>
       <c r="C683" t="inlineStr">
         <is>
-          <t>GIFT BAG HOLOGRAPH 18X23CM MED1920</t>
+          <t>GIFT BAG NON-WOVEN PRINTED Asst</t>
         </is>
       </c>
       <c r="D683" s="2" t="n">
-        <v>324</v>
+        <v>9</v>
       </c>
       <c r="E683" s="3" t="n">
-        <v>1920</v>
+        <v>8656</v>
       </c>
       <c r="F683" t="inlineStr">
         <is>
@@ -21303,7 +21303,7 @@
         </is>
       </c>
       <c r="D749" s="2" t="n">
-        <v>507</v>
+        <v>495</v>
       </c>
       <c r="E749" s="3" t="n">
         <v>13106</v>
@@ -22031,7 +22031,7 @@
         </is>
       </c>
       <c r="D775" s="2" t="n">
-        <v>664</v>
+        <v>628</v>
       </c>
       <c r="E775" s="3" t="n">
         <v>15899</v>
@@ -23207,7 +23207,7 @@
         </is>
       </c>
       <c r="D817" s="2" t="n">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="E817" s="3" t="n">
         <v>16983</v>
@@ -37073,7 +37073,7 @@
         </is>
       </c>
       <c r="D1312" s="2" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E1312" s="3" t="n">
         <v>18577</v>
@@ -39705,7 +39705,7 @@
         </is>
       </c>
       <c r="D1406" s="2" t="n">
-        <v>1978</v>
+        <v>1954</v>
       </c>
       <c r="E1406" s="3" t="n">
         <v>11094</v>
@@ -39733,7 +39733,7 @@
         </is>
       </c>
       <c r="D1407" s="2" t="n">
-        <v>1817</v>
+        <v>1805</v>
       </c>
       <c r="E1407" s="3" t="n">
         <v>10548</v>
@@ -39761,7 +39761,7 @@
         </is>
       </c>
       <c r="D1408" s="2" t="n">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E1408" s="3" t="n">
         <v>15697</v>
@@ -39901,7 +39901,7 @@
         </is>
       </c>
       <c r="D1413" s="2" t="n">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="E1413" s="3" t="n">
         <v>8626</v>
@@ -41049,7 +41049,7 @@
         </is>
       </c>
       <c r="D1454" s="2" t="n">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="E1454" s="3" t="n">
         <v>12419</v>
@@ -42253,7 +42253,7 @@
         </is>
       </c>
       <c r="D1497" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E1497" s="3" t="n">
         <v>37512</v>

</xml_diff>